<commit_message>
Frame the FY2026 scenarios as a nowcast made on 15 Oct 2026 from H1 data
</commit_message>
<xml_diff>
--- a/Shopee_Monee_Unit_Economics.xlsx
+++ b/Shopee_Monee_Unit_Economics.xlsx
@@ -907,7 +907,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Question: is Shopee's growth becoming more profitable, is Monee's fast loan growth staying healthy, and is the 'US$1 billion Shopee adjusted EBITDA in FY2026' expectation realistic?</t>
+          <t>Question: is Shopee's growth becoming more profitable, is Monee's fast loan growth staying healthy, and, before H2 is reported, how likely is the 'US$1 billion Shopee adjusted EBITDA in FY2026' expectation (nowcast as of 15 Oct 2026)?</t>
         </is>
       </c>
     </row>
@@ -6970,7 +6970,7 @@
     <row r="1">
       <c r="A1" s="18" t="inlineStr">
         <is>
-          <t>Can Shopee reach US$1 billion adjusted EBITDA in FY2026?</t>
+          <t>Nowcast: can Shopee reach US$1 billion adjusted EBITDA in FY2026?</t>
         </is>
       </c>
     </row>
@@ -6978,6 +6978,13 @@
       <c r="A2" t="inlineStr">
         <is>
           <t>Sea's CEO said in the Q2 2026 release that he is 'optimistic' Shopee will reach US$1 billion adjusted EBITDA for the full year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Pre-results estimate (nowcast) made on 15 Oct 2026 from H1 2026 data, before Sea reports Q3 2026 (mid-November 2026) and FY2026 (around March 2027).</t>
         </is>
       </c>
     </row>

</xml_diff>